<commit_message>
Updated NW design document
</commit_message>
<xml_diff>
--- a/docs/Design/NW/NW_design_no_tf.xlsx
+++ b/docs/Design/NW/NW_design_no_tf.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ryota/Documents/研鑽/技術/Projects/20250110_KubernetesAPI/graphapp/docs/Design/NW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49496245-6004-9F41-A00C-EA4DE97B7A06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A544C40-8CDA-1F46-802B-308061A7DA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="540" windowWidth="29320" windowHeight="19660" xr2:uid="{A262E15D-8A74-E342-96E0-9E111D7ACA0C}"/>
+    <workbookView xWindow="1400" yWindow="540" windowWidth="29320" windowHeight="19660" activeTab="2" xr2:uid="{A262E15D-8A74-E342-96E0-9E111D7ACA0C}"/>
   </bookViews>
   <sheets>
     <sheet name="System Architecture" sheetId="1" r:id="rId1"/>
     <sheet name="SG_diagram" sheetId="4" r:id="rId2"/>
     <sheet name="SGs" sheetId="2" r:id="rId3"/>
-    <sheet name="EKS" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>System Architecture</t>
   </si>
@@ -72,9 +71,6 @@
   </si>
   <si>
     <t>ALB</t>
-  </si>
-  <si>
-    <t>Worker Nodes and X-ENIs</t>
   </si>
   <si>
     <t>Auto-created and managed by EKS</t>
@@ -125,10 +121,6 @@
     <t>dst</t>
   </si>
   <si>
-    <t>3000
-8080</t>
-  </si>
-  <si>
     <t>Usually auto-created and managed by EKS, but manually create a stricter SG that only permit access from local laptop to ALB.
 Specify with an annotation in ingress.yaml.
 3000: frontend
@@ -138,23 +130,23 @@
     <t>Used in the SG of RDS (No.4) as the src and ALB (No.1) as the dst.</t>
   </si>
   <si>
-    <t>No.1</t>
-  </si>
-  <si>
     <t>No.4</t>
   </si>
   <si>
-    <t>2, 3</t>
+    <t>-</t>
   </si>
   <si>
-    <t>-</t>
+    <t>ALB, Worker Nodes and X-ENIs</t>
+  </si>
+  <si>
+    <t>1, 2, 4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -169,15 +161,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -193,12 +178,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -230,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -249,18 +228,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -10058,7 +10025,7 @@
   <sheetData>
     <row r="3" spans="2:2" ht="32" x14ac:dyDescent="0.4">
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -10085,12 +10052,12 @@
         <v>3</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="2:12" ht="17" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>6</v>
@@ -10099,7 +10066,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>2</v>
@@ -10111,7 +10078,7 @@
         <v>5</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>4</v>
@@ -10128,7 +10095,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>10</v>
@@ -10137,25 +10104,25 @@
         <v>1</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" s="6">
         <v>80</v>
       </c>
-      <c r="I3" s="8" t="s">
-        <v>22</v>
+      <c r="I3" s="6" t="s">
+        <v>30</v>
       </c>
-      <c r="J3" s="8" t="s">
-        <v>8</v>
+      <c r="J3" s="6" t="s">
+        <v>30</v>
       </c>
-      <c r="K3" s="9" t="s">
-        <v>28</v>
+      <c r="K3" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="2:12" ht="17" x14ac:dyDescent="0.2">
@@ -10163,34 +10130,34 @@
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="K4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="34" x14ac:dyDescent="0.2">
@@ -10198,25 +10165,25 @@
         <v>3</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" s="6">
         <v>2</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>31</v>
+      <c r="F5" s="6" t="s">
+        <v>30</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>8</v>
+      <c r="G5" s="6" t="s">
+        <v>30</v>
       </c>
-      <c r="H5" s="11" t="s">
-        <v>28</v>
+      <c r="H5" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>8</v>
@@ -10225,7 +10192,7 @@
         <v>3306</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="17" x14ac:dyDescent="0.2">
@@ -10233,7 +10200,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>7</v>
@@ -10242,7 +10209,7 @@
         <v>4</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>8</v>
@@ -10251,16 +10218,16 @@
         <v>3306</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.2">
@@ -10805,13 +10772,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F69323C4-9753-C94A-ACE3-2A78B06B94A2}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated NW design xlsx
</commit_message>
<xml_diff>
--- a/docs/Design/NW/NW_design_no_tf.xlsx
+++ b/docs/Design/NW/NW_design_no_tf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Ryota/Documents/研鑽/技術/Projects/20250110_KubernetesAPI/graphapp/docs/Design/NW/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A544C40-8CDA-1F46-802B-308061A7DA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCD723DB-2E88-8545-9D30-7D73A183973A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1400" yWindow="540" windowWidth="29320" windowHeight="19660" activeTab="2" xr2:uid="{A262E15D-8A74-E342-96E0-9E111D7ACA0C}"/>
+    <workbookView xWindow="2980" yWindow="1340" windowWidth="29320" windowHeight="19660" activeTab="2" xr2:uid="{A262E15D-8A74-E342-96E0-9E111D7ACA0C}"/>
   </bookViews>
   <sheets>
     <sheet name="System Architecture" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="39">
   <si>
     <t>System Architecture</t>
   </si>
@@ -106,9 +105,6 @@
     <t>No.3</t>
   </si>
   <si>
-    <t>(automatically set)</t>
-  </si>
-  <si>
     <t>Allow DB access from EKS Worker Nodes (No.3) to RDS.</t>
   </si>
   <si>
@@ -136,10 +132,31 @@
     <t>-</t>
   </si>
   <si>
-    <t>ALB, Worker Nodes and X-ENIs</t>
+    <t>1, 2, 4</t>
   </si>
   <si>
-    <t>1, 2, 4</t>
+    <t>eks-cluster-sg-graphapp-eks-cluster-xxxxxxxxxxx</t>
+  </si>
+  <si>
+    <t>eksctl-graphapp-eks-cluster-cluster-ClusterSharedNodeSecurityGroup-xxxxxxxxxxx</t>
+  </si>
+  <si>
+    <t>Automatically created by EKS but not used as the SG No.3 is used instead</t>
+  </si>
+  <si>
+    <t>eksctl-graphapp-eks-cluster-cluster-ControlPlaneSecurityGroup-xxxxxxxxxxx</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>k8s-traffic-graphappekscluster-xxxxxxxxxxx</t>
+  </si>
+  <si>
+    <t>Control plane X-ENIs</t>
+  </si>
+  <si>
+    <t>ALB, Worker Nodes and Control plane X-ENIs</t>
   </si>
 </sst>
 </file>
@@ -162,7 +179,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,13 +188,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -209,25 +232,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -10025,7 +10057,7 @@
   <sheetData>
     <row r="3" spans="2:2" ht="32" x14ac:dyDescent="0.4">
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -10039,735 +10071,796 @@
   <dimension ref="B1:L42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.83203125" style="4"/>
-    <col min="3" max="3" width="60" style="4" customWidth="1"/>
-    <col min="4" max="5" width="23.5" style="4" customWidth="1"/>
-    <col min="6" max="11" width="10.83203125" style="4"/>
-    <col min="12" max="12" width="51.33203125" style="5" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="4"/>
+    <col min="1" max="2" width="10.83203125" style="2"/>
+    <col min="3" max="3" width="60" style="2" customWidth="1"/>
+    <col min="4" max="5" width="23.5" style="2" customWidth="1"/>
+    <col min="6" max="11" width="10.83203125" style="2"/>
+    <col min="12" max="12" width="51.33203125" style="3" customWidth="1"/>
+    <col min="13" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>25</v>
+      <c r="I1" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="2:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="6" t="s">
+      <c r="E2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="J2" s="6" t="s">
+      <c r="I2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="102" x14ac:dyDescent="0.2">
-      <c r="B3" s="6">
+      <c r="B3" s="4">
         <v>1</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="4">
         <v>1</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="4">
         <v>80</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>27</v>
+      <c r="I3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="2:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="B4" s="6">
+      <c r="B4" s="4">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="D4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="34" x14ac:dyDescent="0.2">
-      <c r="B5" s="6">
+      <c r="B5" s="4">
         <v>3</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="4">
         <v>2</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I5" s="6" t="s">
+      <c r="F5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="G5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="4">
         <v>3306</v>
       </c>
-      <c r="L5" s="7" t="s">
-        <v>28</v>
+      <c r="L5" s="5" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="17" x14ac:dyDescent="0.2">
-      <c r="B6" s="6">
+      <c r="B6" s="4">
         <v>4</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="4">
+        <v>3</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="4">
+        <v>3306</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="34" x14ac:dyDescent="0.2">
+      <c r="B7" s="4">
+        <v>5</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="B8" s="4">
+        <v>6</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="9">
         <v>4</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="6">
-        <v>3306</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="L6" s="7" t="s">
-        <v>23</v>
+      <c r="F8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L8" s="10" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B7" s="6">
-        <v>5</v>
-      </c>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="7"/>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B8" s="6">
-        <v>6</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="7"/>
-    </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B9" s="6">
+    <row r="9" spans="2:12" ht="17" x14ac:dyDescent="0.2">
+      <c r="B9" s="4">
         <v>7</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="7"/>
+      <c r="C9" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="L9" s="10" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B10" s="6">
+      <c r="B10" s="4">
         <v>8</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="7"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="5"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B11" s="6">
+      <c r="B11" s="4">
         <v>9</v>
       </c>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="7"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="5"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B12" s="6">
+      <c r="B12" s="4">
         <v>10</v>
       </c>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="7"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="5"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B13" s="6">
+      <c r="B13" s="4">
         <v>11</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="7"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="5"/>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B14" s="6">
+      <c r="B14" s="4">
         <v>12</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="7"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="5"/>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B15" s="6">
+      <c r="B15" s="4">
         <v>13</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="7"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="5"/>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B16" s="6">
+      <c r="B16" s="4">
         <v>14</v>
       </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="7"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="5"/>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B17" s="6">
+      <c r="B17" s="4">
         <v>15</v>
       </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="7"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="5"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B18" s="6">
+      <c r="B18" s="4">
         <v>16</v>
       </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="7"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="5"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B19" s="6">
+      <c r="B19" s="4">
         <v>17</v>
       </c>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="7"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="5"/>
     </row>
     <row r="20" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B20" s="6">
+      <c r="B20" s="4">
         <v>18</v>
       </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="7"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="5"/>
     </row>
     <row r="21" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B21" s="6">
+      <c r="B21" s="4">
         <v>19</v>
       </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="7"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="5"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B22" s="6">
+      <c r="B22" s="4">
         <v>20</v>
       </c>
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="7"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="5"/>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B23" s="6">
+      <c r="B23" s="4">
         <v>21</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
-      <c r="L23" s="7"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="5"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B24" s="6">
+      <c r="B24" s="4">
         <v>22</v>
       </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6"/>
-      <c r="L24" s="7"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="5"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B25" s="6">
+      <c r="B25" s="4">
         <v>23</v>
       </c>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="7"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="5"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B26" s="6">
+      <c r="B26" s="4">
         <v>24</v>
       </c>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="7"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="5"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B27" s="6">
+      <c r="B27" s="4">
         <v>25</v>
       </c>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="7"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="5"/>
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B28" s="6">
+      <c r="B28" s="4">
         <v>26</v>
       </c>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="7"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="5"/>
     </row>
     <row r="29" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B29" s="6">
+      <c r="B29" s="4">
         <v>27</v>
       </c>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="7"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="5"/>
     </row>
     <row r="30" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B30" s="6">
+      <c r="B30" s="4">
         <v>28</v>
       </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="7"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="5"/>
     </row>
     <row r="31" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B31" s="6">
+      <c r="B31" s="4">
         <v>29</v>
       </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="7"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
+      <c r="L31" s="5"/>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B32" s="6">
+      <c r="B32" s="4">
         <v>30</v>
       </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="7"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="5"/>
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B33" s="6">
+      <c r="B33" s="4">
         <v>31</v>
       </c>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="6"/>
-      <c r="L33" s="7"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="5"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B34" s="6">
+      <c r="B34" s="4">
         <v>32</v>
       </c>
-      <c r="C34" s="6"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6"/>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="6"/>
-      <c r="K34" s="6"/>
-      <c r="L34" s="7"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="5"/>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B35" s="6">
+      <c r="B35" s="4">
         <v>33</v>
       </c>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6"/>
-      <c r="E35" s="6"/>
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
-      <c r="L35" s="7"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
+      <c r="K35" s="4"/>
+      <c r="L35" s="5"/>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B36" s="6">
+      <c r="B36" s="4">
         <v>34</v>
       </c>
-      <c r="C36" s="6"/>
-      <c r="D36" s="6"/>
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="6"/>
-      <c r="K36" s="6"/>
-      <c r="L36" s="7"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+      <c r="I36" s="4"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="5"/>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="6">
+      <c r="B37" s="4">
         <v>35</v>
       </c>
-      <c r="C37" s="6"/>
-      <c r="D37" s="6"/>
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="6"/>
-      <c r="K37" s="6"/>
-      <c r="L37" s="7"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
+      <c r="I37" s="4"/>
+      <c r="J37" s="4"/>
+      <c r="K37" s="4"/>
+      <c r="L37" s="5"/>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B38" s="6">
+      <c r="B38" s="4">
         <v>36</v>
       </c>
-      <c r="C38" s="6"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="6"/>
-      <c r="K38" s="6"/>
-      <c r="L38" s="7"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
+      <c r="I38" s="4"/>
+      <c r="J38" s="4"/>
+      <c r="K38" s="4"/>
+      <c r="L38" s="5"/>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B39" s="6">
+      <c r="B39" s="4">
         <v>37</v>
       </c>
-      <c r="C39" s="6"/>
-      <c r="D39" s="6"/>
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="7"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="5"/>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B40" s="6">
+      <c r="B40" s="4">
         <v>38</v>
       </c>
-      <c r="C40" s="6"/>
-      <c r="D40" s="6"/>
-      <c r="E40" s="6"/>
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
-      <c r="J40" s="6"/>
-      <c r="K40" s="6"/>
-      <c r="L40" s="7"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="4"/>
+      <c r="L40" s="5"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B41" s="6">
+      <c r="B41" s="4">
         <v>39</v>
       </c>
-      <c r="C41" s="6"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="6"/>
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="6"/>
-      <c r="K41" s="6"/>
-      <c r="L41" s="7"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="4"/>
+      <c r="L41" s="5"/>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B42" s="6">
+      <c r="B42" s="4">
         <v>40</v>
       </c>
-      <c r="C42" s="6"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="6"/>
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="6"/>
-      <c r="K42" s="6"/>
-      <c r="L42" s="7"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="4"/>
+      <c r="L42" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>